<commit_message>
fix: update frontend server to python3 http.server and fix driver factory
</commit_message>
<xml_diff>
--- a/selenium-tests/reports/E2E_Report.xlsx
+++ b/selenium-tests/reports/E2E_Report.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="210">
   <si>
     <t>Metric Parameter</t>
   </si>
@@ -25,7 +25,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 10:09:46 am</t>
+    <t>28/7/2026, 10:53:53 am</t>
   </si>
   <si>
     <t>Environment</t>
@@ -55,52 +55,388 @@
     <t>Pass Percentage</t>
   </si>
   <si>
-    <t>100.00%</t>
+    <t>51.52%</t>
   </si>
   <si>
     <t>Execution Duration (sec)</t>
   </si>
   <si>
+    <t>90.91s</t>
+  </si>
+  <si>
+    <t>Test ID</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>Scenario Name</t>
+  </si>
+  <si>
+    <t>Browser</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Start Time</t>
+  </si>
+  <si>
+    <t>End Time</t>
+  </si>
+  <si>
+    <t>Duration</t>
+  </si>
+  <si>
+    <t>TC_300</t>
+  </si>
+  <si>
+    <t>AUTH</t>
+  </si>
+  <si>
+    <t>Authentication &amp; Session E2E Test Suite AUTH_01: Validate login form with empty username and password</t>
+  </si>
+  <si>
+    <t>PASSED</t>
+  </si>
+  <si>
+    <t>10:52:50 am</t>
+  </si>
+  <si>
+    <t>10:52:55 am</t>
+  </si>
+  <si>
+    <t>4.85s</t>
+  </si>
+  <si>
+    <t>TC_478</t>
+  </si>
+  <si>
+    <t>FAILED</t>
+  </si>
+  <si>
+    <t>10:52:58 am</t>
+  </si>
+  <si>
+    <t>2.48s</t>
+  </si>
+  <si>
+    <t>TC_724</t>
+  </si>
+  <si>
+    <t>Authentication &amp; Session E2E Test Suite AUTH_02: Validate login rejection with invalid credentials</t>
+  </si>
+  <si>
+    <t>10:53:00 am</t>
+  </si>
+  <si>
+    <t>2.20s</t>
+  </si>
+  <si>
+    <t>TC_362</t>
+  </si>
+  <si>
+    <t>10:53:03 am</t>
+  </si>
+  <si>
+    <t>2.53s</t>
+  </si>
+  <si>
+    <t>TC_372</t>
+  </si>
+  <si>
+    <t>Authentication &amp; Session E2E Test Suite AUTH_03: Validate successful Donor login and role-based redirect</t>
+  </si>
+  <si>
+    <t>10:53:07 am</t>
+  </si>
+  <si>
+    <t>4.42s</t>
+  </si>
+  <si>
+    <t>TC_299</t>
+  </si>
+  <si>
+    <t>10:53:10 am</t>
+  </si>
+  <si>
+    <t>2.68s</t>
+  </si>
+  <si>
+    <t>TC_803</t>
+  </si>
+  <si>
+    <t>Authentication &amp; Session E2E Test Suite AUTH_04: Validate session persistence upon page refresh</t>
+  </si>
+  <si>
+    <t>10:53:12 am</t>
+  </si>
+  <si>
+    <t>1.98s</t>
+  </si>
+  <si>
+    <t>TC_330</t>
+  </si>
+  <si>
+    <t>0.38s</t>
+  </si>
+  <si>
+    <t>TC_898</t>
+  </si>
+  <si>
+    <t>Authentication &amp; Session E2E Test Suite AUTH_05: Validate successful Donor Logout</t>
+  </si>
+  <si>
+    <t>10:53:17 am</t>
+  </si>
+  <si>
+    <t>5.04s</t>
+  </si>
+  <si>
+    <t>TC_792</t>
+  </si>
+  <si>
+    <t>Authentication &amp; Session E2E Test Suite AUTH_06: Validate protected donor route redirects unauthenticated user</t>
+  </si>
+  <si>
+    <t>10:53:20 am</t>
+  </si>
+  <si>
+    <t>2.36s</t>
+  </si>
+  <si>
+    <t>TC_597</t>
+  </si>
+  <si>
+    <t>0.25s</t>
+  </si>
+  <si>
+    <t>TC_453</t>
+  </si>
+  <si>
+    <t>Authentication &amp; Session E2E Test Suite AUTH_07: Validate successful Receiver login and role-based redirect</t>
+  </si>
+  <si>
+    <t>10:53:22 am</t>
+  </si>
+  <si>
+    <t>2.03s</t>
+  </si>
+  <si>
+    <t>TC_426</t>
+  </si>
+  <si>
+    <t>10:53:24 am</t>
+  </si>
+  <si>
+    <t>2.37s</t>
+  </si>
+  <si>
+    <t>TC_840</t>
+  </si>
+  <si>
+    <t>FORMS</t>
+  </si>
+  <si>
+    <t>Form Validation &amp; Input Rules E2E Test Suite FORM_01: Validate Registration form required fields validation</t>
+  </si>
+  <si>
+    <t>10:53:25 am</t>
+  </si>
+  <si>
+    <t>TC_366</t>
+  </si>
+  <si>
+    <t>10:53:27 am</t>
+  </si>
+  <si>
+    <t>2.15s</t>
+  </si>
+  <si>
+    <t>TC_932</t>
+  </si>
+  <si>
+    <t>Form Validation &amp; Input Rules E2E Test Suite FORM_02: Validate Registration email format constraints</t>
+  </si>
+  <si>
+    <t>10:53:29 am</t>
+  </si>
+  <si>
+    <t>2.35s</t>
+  </si>
+  <si>
+    <t>TC_434</t>
+  </si>
+  <si>
+    <t>10:53:30 am</t>
+  </si>
+  <si>
+    <t>0.16s</t>
+  </si>
+  <si>
+    <t>TC_225</t>
+  </si>
+  <si>
+    <t>Form Validation &amp; Input Rules E2E Test Suite FORM_03: Validate Registration field minimum length rules</t>
+  </si>
+  <si>
+    <t>10:53:32 am</t>
+  </si>
+  <si>
+    <t>2.11s</t>
+  </si>
+  <si>
+    <t>TC_665</t>
+  </si>
+  <si>
+    <t>0.26s</t>
+  </si>
+  <si>
+    <t>TC_189</t>
+  </si>
+  <si>
+    <t>Form Validation &amp; Input Rules E2E Test Suite FORM_04: Validate Food Listing form inputs validation rules</t>
+  </si>
+  <si>
+    <t>10:53:34 am</t>
+  </si>
+  <si>
+    <t>2.00s</t>
+  </si>
+  <si>
+    <t>TC_515</t>
+  </si>
+  <si>
+    <t>10:53:36 am</t>
+  </si>
+  <si>
+    <t>TC_376</t>
+  </si>
+  <si>
+    <t>UI-NAVIGATION</t>
+  </si>
+  <si>
+    <t>UI Components &amp; Navigation E2E Test Suite NAV_01: Validate public navbar navigation links</t>
+  </si>
+  <si>
+    <t>10:53:37 am</t>
+  </si>
+  <si>
+    <t>0.30s</t>
+  </si>
+  <si>
+    <t>TC_231</t>
+  </si>
+  <si>
+    <t>10:53:39 am</t>
+  </si>
+  <si>
+    <t>2.38s</t>
+  </si>
+  <si>
+    <t>UI Components &amp; Navigation E2E Test Suite NAV_02: Validate browser back and forward history actions</t>
+  </si>
+  <si>
+    <t>10:53:41 am</t>
+  </si>
+  <si>
+    <t>2.07s</t>
+  </si>
+  <si>
+    <t>TC_170</t>
+  </si>
+  <si>
+    <t>10:53:42 am</t>
+  </si>
+  <si>
+    <t>0.32s</t>
+  </si>
+  <si>
+    <t>TC_329</t>
+  </si>
+  <si>
+    <t>UI Components &amp; Navigation E2E Test Suite UI_01: Validate Receiver Feed search bar and category filters</t>
+  </si>
+  <si>
+    <t>10:53:44 am</t>
+  </si>
+  <si>
+    <t>1.83s</t>
+  </si>
+  <si>
+    <t>TC_334</t>
+  </si>
+  <si>
+    <t>0.56s</t>
+  </si>
+  <si>
+    <t>TC_995</t>
+  </si>
+  <si>
+    <t>DYNAMIC-DISCOVERY</t>
+  </si>
+  <si>
+    <t>Dynamic React Route &amp; Form Discovery Test Suite DYN_01: Verify all discovered React routes are accessible or enforce protection</t>
+  </si>
+  <si>
+    <t>10:53:46 am</t>
+  </si>
+  <si>
+    <t>1.67s</t>
+  </si>
+  <si>
+    <t>TC_993</t>
+  </si>
+  <si>
+    <t>10:53:47 am</t>
+  </si>
+  <si>
+    <t>0.71s</t>
+  </si>
+  <si>
+    <t>TC_295</t>
+  </si>
+  <si>
+    <t>Dynamic React Route &amp; Form Discovery Test Suite DYN_02: Execute dynamically generated test cases from form analysis</t>
+  </si>
+  <si>
+    <t>10:53:48 am</t>
+  </si>
+  <si>
+    <t>1.56s</t>
+  </si>
+  <si>
+    <t>TC_379</t>
+  </si>
+  <si>
+    <t>10:53:49 am</t>
+  </si>
+  <si>
+    <t>0.82s</t>
+  </si>
+  <si>
+    <t>TC_168</t>
+  </si>
+  <si>
+    <t>E2E-WORKFLOW</t>
+  </si>
+  <si>
+    <t>Complete End-to-End Business Workflow Test Suite E2E_01: Complete Donor Publishing to Receiver Claiming &amp; Verification Workflow</t>
+  </si>
+  <si>
+    <t>10:53:51 am</t>
+  </si>
+  <si>
     <t>1.45s</t>
   </si>
   <si>
-    <t>Test ID</t>
-  </si>
-  <si>
-    <t>Module</t>
-  </si>
-  <si>
-    <t>Scenario Name</t>
-  </si>
-  <si>
-    <t>Browser</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Start Time</t>
-  </si>
-  <si>
-    <t>End Time</t>
-  </si>
-  <si>
-    <t>Duration</t>
-  </si>
-  <si>
-    <t>TC_101</t>
-  </si>
-  <si>
-    <t>AUTHENTICATION</t>
-  </si>
-  <si>
-    <t>AUTH_03: Validate successful Donor login</t>
-  </si>
-  <si>
-    <t>PASSED</t>
-  </si>
-  <si>
-    <t>10:09:46 am</t>
+    <t>TC_891</t>
+  </si>
+  <si>
+    <t>10:53:52 am</t>
+  </si>
+  <si>
+    <t>0.93s</t>
   </si>
   <si>
     <t>Test Name</t>
@@ -115,6 +451,76 @@
     <t>URL</t>
   </si>
   <si>
+    <t xml:space="preserve">unknown error: net::ERR_CONNECTION_REFUSED
+  (Session info: chrome=150.0.7871.187)</t>
+  </si>
+  <si>
+    <t>C:\Users\HP\Downloads\SHAREBITE-main\selenium-tests\reports\failures\FAIL_Authentication___Session_E2E_Test_Suite_AUTH_01__Validate_login_form_with_empty_username_and_password_2026-07-28T05-22-58-107Z.png</t>
+  </si>
+  <si>
+    <t>http://localhost:5173/login</t>
+  </si>
+  <si>
+    <t>C:\Users\HP\Downloads\SHAREBITE-main\selenium-tests\reports\failures\FAIL_Authentication___Session_E2E_Test_Suite_AUTH_02__Validate_login_rejection_with_invalid_credentials_2026-07-28T05-23-02-916Z.png</t>
+  </si>
+  <si>
+    <t>C:\Users\HP\Downloads\SHAREBITE-main\selenium-tests\reports\failures\FAIL_Authentication___Session_E2E_Test_Suite_AUTH_03__Validate_successful_Donor_login_and_role-based_redirect_2026-07-28T05-23-10-131Z.png</t>
+  </si>
+  <si>
+    <t>expected 'http://localhost:5173/login' to include '/donor'</t>
+  </si>
+  <si>
+    <t>C:\Users\HP\Downloads\SHAREBITE-main\selenium-tests\reports\failures\FAIL_Authentication___Session_E2E_Test_Suite_AUTH_04__Validate_session_persistence_upon_page_refresh_2026-07-28T05-23-12-567Z.png</t>
+  </si>
+  <si>
+    <t>C:\Users\HP\Downloads\SHAREBITE-main\selenium-tests\reports\failures\FAIL_Authentication___Session_E2E_Test_Suite_AUTH_06__Validate_protected_donor_route_redirects_unauthenticated_user_2026-07-28T05-23-20-285Z.png</t>
+  </si>
+  <si>
+    <t>http://localhost:5173/donor/overview</t>
+  </si>
+  <si>
+    <t>C:\Users\HP\Downloads\SHAREBITE-main\selenium-tests\reports\failures\FAIL_Authentication___Session_E2E_Test_Suite_AUTH_07__Validate_successful_Receiver_login_and_role-based_redirect_2026-07-28T05-23-24-767Z.png</t>
+  </si>
+  <si>
+    <t>C:\Users\HP\Downloads\SHAREBITE-main\selenium-tests\reports\failures\FAIL_Form_Validation___Input_Rules_E2E_Test_Suite_FORM_01__Validate_Registration_form_required_fields_validation_2026-07-28T05-23-27-246Z.png</t>
+  </si>
+  <si>
+    <t>http://localhost:5173/register</t>
+  </si>
+  <si>
+    <t>C:\Users\HP\Downloads\SHAREBITE-main\selenium-tests\reports\failures\FAIL_Form_Validation___Input_Rules_E2E_Test_Suite_FORM_02__Validate_Registration_email_format_constraints_2026-07-28T05-23-29-900Z.png</t>
+  </si>
+  <si>
+    <t>C:\Users\HP\Downloads\SHAREBITE-main\selenium-tests\reports\failures\FAIL_Form_Validation___Input_Rules_E2E_Test_Suite_FORM_03__Validate_Registration_field_minimum_length_rules_2026-07-28T05-23-32-380Z.png</t>
+  </si>
+  <si>
+    <t>C:\Users\HP\Downloads\SHAREBITE-main\selenium-tests\reports\failures\FAIL_Form_Validation___Input_Rules_E2E_Test_Suite_FORM_04__Validate_Food_Listing_form_inputs_validation_rules_2026-07-28T05-23-36-859Z.png</t>
+  </si>
+  <si>
+    <t>C:\Users\HP\Downloads\SHAREBITE-main\selenium-tests\reports\failures\FAIL_UI_Components___Navigation_E2E_Test_Suite_NAV_01__Validate_public_navbar_navigation_links_2026-07-28T05-23-39-636Z.png</t>
+  </si>
+  <si>
+    <t>http://localhost:5173/</t>
+  </si>
+  <si>
+    <t>expected 'http://localhost:5173/register' to include '/platform'</t>
+  </si>
+  <si>
+    <t>C:\Users\HP\Downloads\SHAREBITE-main\selenium-tests\reports\failures\FAIL_UI_Components___Navigation_E2E_Test_Suite_NAV_02__Validate_browser_back_and_forward_history_actions_2026-07-28T05-23-42-130Z.png</t>
+  </si>
+  <si>
+    <t>C:\Users\HP\Downloads\SHAREBITE-main\selenium-tests\reports\failures\FAIL_UI_Components___Navigation_E2E_Test_Suite_UI_01__Validate_Receiver_Feed_search_bar_and_category_filters_2026-07-28T05-23-44-774Z.png</t>
+  </si>
+  <si>
+    <t>C:\Users\HP\Downloads\SHAREBITE-main\selenium-tests\reports\failures\FAIL_Dynamic_React_Route___Form_Discovery_Test_Suite_DYN_01__Verify_all_discovered_React_routes_are_accessible_or_enforce_protection_2026-07-28T05-23-47-290Z.png</t>
+  </si>
+  <si>
+    <t>C:\Users\HP\Downloads\SHAREBITE-main\selenium-tests\reports\failures\FAIL_Dynamic_React_Route___Form_Discovery_Test_Suite_DYN_02__Execute_dynamically_generated_test_cases_from_form_analysis_2026-07-28T05-23-49-825Z.png</t>
+  </si>
+  <si>
+    <t>C:\Users\HP\Downloads\SHAREBITE-main\selenium-tests\reports\failures\FAIL_Complete_End-to-End_Business_Workflow_Test_Suite_E2E_01__Complete_Donor_Publishing_to_Receiver_Claiming___Verification_Workflow_2026-07-28T05-23-52-341Z.png</t>
+  </si>
+  <si>
     <t>Timestamp</t>
   </si>
   <si>
@@ -127,17 +533,126 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>Direct CLI report generation check</t>
-  </si>
-  <si>
-    <t>Baseline Excel report compiled</t>
+    <t>28/7/2026, 10:52:55 am</t>
+  </si>
+  <si>
+    <t>Execution of test step in auth</t>
+  </si>
+  <si>
+    <t>Completed successfully</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:52:58 am</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Failed: unknown error: net::ERR_CONNECTION_REFUSED
+  (Session info: chrome=150.0.7871.187)</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:00 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:03 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:07 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:10 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:12 am</t>
+  </si>
+  <si>
+    <t>Failed: expected 'http://localhost:5173/login' to include '/donor'</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:17 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:20 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:22 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:24 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:25 am</t>
+  </si>
+  <si>
+    <t>Execution of test step in forms</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:27 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:29 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:30 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:32 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:34 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:36 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:37 am</t>
+  </si>
+  <si>
+    <t>Execution of test step in ui-navigation</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:39 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:41 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:42 am</t>
+  </si>
+  <si>
+    <t>Failed: expected 'http://localhost:5173/register' to include '/platform'</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:44 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:46 am</t>
+  </si>
+  <si>
+    <t>Execution of test step in dynamic-discovery</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:47 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:48 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:49 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:51 am</t>
+  </si>
+  <si>
+    <t>Execution of test step in e2e-workflow</t>
+  </si>
+  <si>
+    <t>28/7/2026, 10:53:52 am</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -155,8 +670,12 @@
       <b/>
       <color rgb="15803D"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="B91C1C"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -171,6 +690,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="DCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FEE2E2"/>
       </patternFill>
     </fill>
   </fills>
@@ -201,11 +725,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -589,7 +1114,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="2">
-        <v>1</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -597,7 +1122,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="2">
-        <v>1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -605,7 +1130,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="2">
-        <v>0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -640,7 +1165,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -697,10 +1222,842 @@
         <v>28</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>15</v>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -711,7 +2068,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
@@ -723,19 +2080,291 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>141</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>142</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>31</v>
+        <v>143</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>32</v>
+        <v>144</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -746,7 +2375,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -758,36 +2387,580 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>168</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>141</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>34</v>
+        <v>169</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>35</v>
+        <v>170</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>36</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>172</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>37</v>
+        <v>173</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>38</v>
+        <v>174</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: restore all test suites and github action workflows
</commit_message>
<xml_diff>
--- a/selenium-tests/reports/E2E_Report.xlsx
+++ b/selenium-tests/reports/E2E_Report.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="129">
   <si>
     <t>Metric Parameter</t>
   </si>
@@ -25,7 +25,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 11:37:19 am</t>
+    <t>28/7/2026, 11:45:33 am</t>
   </si>
   <si>
     <t>Environment</t>
@@ -61,7 +61,7 @@
     <t>Execution Duration (sec)</t>
   </si>
   <si>
-    <t>1.45s</t>
+    <t>176.76s</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -88,19 +88,229 @@
     <t>Duration</t>
   </si>
   <si>
-    <t>TC_101</t>
-  </si>
-  <si>
-    <t>AUTHENTICATION</t>
-  </si>
-  <si>
-    <t>AUTH_03: Validate successful Donor login</t>
+    <t>TC_594</t>
+  </si>
+  <si>
+    <t>AUTH</t>
+  </si>
+  <si>
+    <t>Authentication &amp; Session E2E Test Suite AUTH_01: Validate login form with empty username and password</t>
   </si>
   <si>
     <t>PASSED</t>
   </si>
   <si>
-    <t>11:37:19 am</t>
+    <t>11:42:37 am</t>
+  </si>
+  <si>
+    <t>11:42:47 am</t>
+  </si>
+  <si>
+    <t>9.80s</t>
+  </si>
+  <si>
+    <t>TC_975</t>
+  </si>
+  <si>
+    <t>Authentication &amp; Session E2E Test Suite AUTH_02: Validate login rejection with invalid credentials</t>
+  </si>
+  <si>
+    <t>11:42:57 am</t>
+  </si>
+  <si>
+    <t>9.74s</t>
+  </si>
+  <si>
+    <t>TC_140</t>
+  </si>
+  <si>
+    <t>Authentication &amp; Session E2E Test Suite AUTH_03: Validate successful Donor login and role-based redirect</t>
+  </si>
+  <si>
+    <t>11:43:04 am</t>
+  </si>
+  <si>
+    <t>7.40s</t>
+  </si>
+  <si>
+    <t>TC_309</t>
+  </si>
+  <si>
+    <t>Authentication &amp; Session E2E Test Suite AUTH_04: Validate session persistence upon page refresh</t>
+  </si>
+  <si>
+    <t>11:43:07 am</t>
+  </si>
+  <si>
+    <t>2.38s</t>
+  </si>
+  <si>
+    <t>TC_886</t>
+  </si>
+  <si>
+    <t>Authentication &amp; Session E2E Test Suite AUTH_05: Validate successful Donor Logout</t>
+  </si>
+  <si>
+    <t>11:43:12 am</t>
+  </si>
+  <si>
+    <t>5.04s</t>
+  </si>
+  <si>
+    <t>TC_340</t>
+  </si>
+  <si>
+    <t>Authentication &amp; Session E2E Test Suite AUTH_06: Validate protected donor route redirects unauthenticated user</t>
+  </si>
+  <si>
+    <t>11:43:14 am</t>
+  </si>
+  <si>
+    <t>2.37s</t>
+  </si>
+  <si>
+    <t>TC_206</t>
+  </si>
+  <si>
+    <t>Authentication &amp; Session E2E Test Suite AUTH_07: Validate successful Receiver login and role-based redirect</t>
+  </si>
+  <si>
+    <t>11:43:19 am</t>
+  </si>
+  <si>
+    <t>5.29s</t>
+  </si>
+  <si>
+    <t>TC_418</t>
+  </si>
+  <si>
+    <t>FORMS</t>
+  </si>
+  <si>
+    <t>Form Validation &amp; Input Rules E2E Test Suite FORM_01: Validate Registration form required fields validation</t>
+  </si>
+  <si>
+    <t>11:43:27 am</t>
+  </si>
+  <si>
+    <t>7.39s</t>
+  </si>
+  <si>
+    <t>TC_197</t>
+  </si>
+  <si>
+    <t>Form Validation &amp; Input Rules E2E Test Suite FORM_02: Validate Registration email format constraints</t>
+  </si>
+  <si>
+    <t>11:43:37 am</t>
+  </si>
+  <si>
+    <t>9.75s</t>
+  </si>
+  <si>
+    <t>TC_650</t>
+  </si>
+  <si>
+    <t>Form Validation &amp; Input Rules E2E Test Suite FORM_03: Validate Registration field minimum length rules</t>
+  </si>
+  <si>
+    <t>11:43:44 am</t>
+  </si>
+  <si>
+    <t>7.44s</t>
+  </si>
+  <si>
+    <t>TC_549</t>
+  </si>
+  <si>
+    <t>Form Validation &amp; Input Rules E2E Test Suite FORM_04: Validate Food Listing form inputs validation rules</t>
+  </si>
+  <si>
+    <t>11:43:59 am</t>
+  </si>
+  <si>
+    <t>14.80s</t>
+  </si>
+  <si>
+    <t>TC_865</t>
+  </si>
+  <si>
+    <t>UI-NAVIGATION</t>
+  </si>
+  <si>
+    <t>UI Components &amp; Navigation E2E Test Suite NAV_01: Validate public navbar navigation links</t>
+  </si>
+  <si>
+    <t>11:44:06 am</t>
+  </si>
+  <si>
+    <t>7.43s</t>
+  </si>
+  <si>
+    <t>TC_731</t>
+  </si>
+  <si>
+    <t>UI Components &amp; Navigation E2E Test Suite NAV_02: Validate browser back and forward history actions</t>
+  </si>
+  <si>
+    <t>11:44:09 am</t>
+  </si>
+  <si>
+    <t>2.65s</t>
+  </si>
+  <si>
+    <t>TC_280</t>
+  </si>
+  <si>
+    <t>UI Components &amp; Navigation E2E Test Suite UI_01: Validate Receiver Feed search bar and category filters</t>
+  </si>
+  <si>
+    <t>11:44:23 am</t>
+  </si>
+  <si>
+    <t>14.57s</t>
+  </si>
+  <si>
+    <t>TC_592</t>
+  </si>
+  <si>
+    <t>DYNAMIC-DISCOVERY</t>
+  </si>
+  <si>
+    <t>Dynamic React Route &amp; Form Discovery Test Suite DYN_01: Verify all discovered React routes are accessible or enforce protection</t>
+  </si>
+  <si>
+    <t>11:44:31 am</t>
+  </si>
+  <si>
+    <t>7.11s</t>
+  </si>
+  <si>
+    <t>TC_329</t>
+  </si>
+  <si>
+    <t>Dynamic React Route &amp; Form Discovery Test Suite DYN_02: Execute dynamically generated test cases from form analysis</t>
+  </si>
+  <si>
+    <t>11:44:36 am</t>
+  </si>
+  <si>
+    <t>5.05s</t>
+  </si>
+  <si>
+    <t>TC_374</t>
+  </si>
+  <si>
+    <t>E2E-WORKFLOW</t>
+  </si>
+  <si>
+    <t>Complete End-to-End Business Workflow Test Suite E2E_01: Complete Donor Publishing to Receiver Claiming &amp; Verification Workflow</t>
+  </si>
+  <si>
+    <t>11:45:33 am</t>
+  </si>
+  <si>
+    <t>57.60s</t>
   </si>
   <si>
     <t>Test Name</t>
@@ -127,10 +337,70 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>Direct CLI report generation check</t>
-  </si>
-  <si>
-    <t>Baseline Excel report compiled</t>
+    <t>28/7/2026, 11:42:47 am</t>
+  </si>
+  <si>
+    <t>Execution of test step in auth</t>
+  </si>
+  <si>
+    <t>Completed successfully</t>
+  </si>
+  <si>
+    <t>28/7/2026, 11:42:57 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 11:43:04 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 11:43:07 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 11:43:12 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 11:43:14 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 11:43:19 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 11:43:27 am</t>
+  </si>
+  <si>
+    <t>Execution of test step in forms</t>
+  </si>
+  <si>
+    <t>28/7/2026, 11:43:37 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 11:43:44 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 11:43:59 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 11:44:06 am</t>
+  </si>
+  <si>
+    <t>Execution of test step in ui-navigation</t>
+  </si>
+  <si>
+    <t>28/7/2026, 11:44:09 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 11:44:23 am</t>
+  </si>
+  <si>
+    <t>28/7/2026, 11:44:31 am</t>
+  </si>
+  <si>
+    <t>Execution of test step in dynamic-discovery</t>
+  </si>
+  <si>
+    <t>28/7/2026, 11:44:36 am</t>
+  </si>
+  <si>
+    <t>Execution of test step in e2e-workflow</t>
   </si>
 </sst>
 </file>
@@ -589,7 +859,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="2">
-        <v>1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -597,7 +867,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="2">
-        <v>1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -640,7 +910,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -697,10 +967,426 @@
         <v>28</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>15</v>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -723,19 +1409,19 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>99</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>31</v>
+        <v>101</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>32</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -746,7 +1432,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -758,36 +1444,308 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>103</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>99</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>34</v>
+        <v>104</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>35</v>
+        <v>105</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>36</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>107</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>37</v>
+        <v>108</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>38</v>
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>